<commit_message>
Example workbooks made by code of their own; no numbered discussion links (#195)
The five example reports are built from new example ARDs and plan code
(the cards example data and made-up values), exercising the same
features and checked the same way; the workbooks are regenerated.  The
docs, tests and NEWS no longer point to discussions by number, and their
examples use neutral variable names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -9,13 +9,15 @@
     <sheet name="study" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="tables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="variables" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="cells" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="layout" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="columns" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="style" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="cell_styles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="col_header" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="about" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="codelists" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="cells" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="digits" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="layout" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="columns" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="style" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="cell_styles" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="col_header" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="about" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -56,6 +58,286 @@
 </comments>
 </file>
 
+<file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tflspec</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The report a row belongs to. Blank: a study-wide default; a row naming a report replaces the default row with the same key (ARD analyses: the report the analysis serves).
+Example: T-14-1-1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The columns styled, | between them (.values = every value column); blank: every column.
+Example: Placebo | .values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: TRUE styles the column header instead of the body; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">An R condition over the table's columns choosing the rows; blank: every row. Two rows with a where may not set the same look: join their conditions with |.
+Example: label == "Any TEAE"</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">left / center / right; blank: unchanged.
+Example: center</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Text colour, #RRGGBB; blank: unchanged.
+Example: #CC0000</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Cell shading, #RRGGBB; blank: unchanged.
+Example: #EEEEEE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Left indent of the cell text in twips (not on the header); blank: unchanged.
+Example: 200</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tflspec</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The report a row belongs to. Blank: a study-wide default; a row naming a report replaces the default row with the same key (ARD analyses: the report the analysis serves).
+Example: T-14-1-1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The header row, a whole number (1 = the top).
+Example: 1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The columns the cell sits on: a name, .values (every value column), a position or range (3, 3:31, 3:last), or KEY = value (the columns whose key has that value); | between them.
+Example: .values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Blank: one cell over cols; each: one cell a column; a key's name: one cell per value of that key (a spanner).
+Example: TR01AG1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">What prints; a line break is Alt+Enter or \n. Tokens: {col} {col1} {col2} (the column's keys), {n} {n1} {n2} (the population at that depth, read from the ARD), {n:sum} (the total over the cell's columns). Quote it to keep leading spaces.
+Example: {col1}\n(N={n:sum})</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">left / center / right (col_cell()); blank: the default.
+Example: center</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The cell's top rule: single / double / none ... (rtf_border()); blank: the header's.
+Example: single</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The cell's bottom rule, as border_top.
+Example: single</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
@@ -135,7 +417,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">With stats = rows: stat (the number) or stat_fmt (cards' formatted text) (plan_cells(value = )); blank: stat.
+          <t xml:space="preserve">Which of the ARD's values the table prints: stat (the number, rounded here: the digits sheet, a template's {x:.1f}) or stat_fmt (the ARD's own text, as it was formatted: no digits to set; a template still combines them, {mean} ({sd})); a row may say otherwise in its template ({mean:stat_fmt}, {mean:.1f}). With stats = rows: which goes in the cell (plan_cells(value = )). Blank: stat.
 Example: stat</t>
         </r>
       </text>
@@ -292,6 +574,19 @@
         </r>
       </text>
     </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Its values no record has -- a code list's value, counted 0 in every column -- show (a 0 row) or hide (plan_levels(.drop_empty = )); blank: show.
+Example: hide</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -323,8 +618,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">What the template is for: a variable, continuous / categorical (every variable of that kind); blank: every variable.
-Example: continuous</t>
+          <t xml:space="preserve">The variable (an analysis variable or a column key).
+Example: SEX</t>
         </r>
       </text>
     </comment>
@@ -336,8 +631,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Only the ARD rows of this context (one variable summarised two ways); blank: any.
-Example: summary</t>
+          <t xml:space="preserve">A value as the data have it.
+Example: F</t>
         </r>
       </text>
     </comment>
@@ -349,8 +644,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The row's label; blank: one row a level, labelled by the level.
-Example: Mean (SD)</t>
+          <t xml:space="preserve">What the value is in the data the program makes, and so what prints; blank: the value.
+Example: Female</t>
         </r>
       </text>
     </comment>
@@ -362,47 +657,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">An R condition on the statistics; the row is used only when it holds; blank: always.
-Example: n == 0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The cell's text with {statistic:format} tokens.
-Example: {mean} ({sd})</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Decimals of a token with no format, a comma between tokens; blank: plan_digits().
-Example: 2,3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Significant digits (wins over digits); blank: none.
-Example: 4</t>
+          <t xml:space="preserve">Its place among the variable's values (a number); blank: after the numbered ones, in the sheet's order.
+Example: 2</t>
         </r>
       </text>
     </comment>
@@ -437,8 +693,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Rows a page (plan_paginate_rows(max_rows = )), a whole number; blank: as_rtftables()' default.
-Example: 26</t>
+          <t xml:space="preserve">What the template is for: a variable, continuous / categorical (every variable of that kind); blank: every variable.
+Example: continuous</t>
         </r>
       </text>
     </comment>
@@ -450,8 +706,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">How a page break may cut: group_safe / group_force / rows / ... (plan_paginate_rows(split = )); blank: as_rtftables()' default.
-Example: group_force</t>
+          <t xml:space="preserve">Only the ARD rows of this context (one variable summarised two ways); blank: any.
+Example: summary</t>
         </r>
       </text>
     </comment>
@@ -463,8 +719,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Row positions to cut before, | between them, with pages_split = rows (plan_paginate_rows(break_before = )); blank: none.
-Example: 20 | 40</t>
+          <t xml:space="preserve">The row's label; blank: one row a level, labelled by the level.
+Example: Mean (SD)</t>
         </r>
       </text>
     </comment>
@@ -476,8 +732,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Rows of a group kept together at the foot of a page, a whole number (plan_paginate_rows(min_group_rows = )); blank: the default.
-Example: 2</t>
+          <t xml:space="preserve">An R condition on the statistics; the row is used only when it holds; blank: always.
+Example: n == 0</t>
         </r>
       </text>
     </comment>
@@ -489,8 +745,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Appended to a group label continued on the next page (plan_paginate_rows(cont_label = )); quote it to keep leading spaces; blank: none.
-Example: " (Cont.)"</t>
+          <t xml:space="preserve">The cell's text with {statistic:format} tokens.
+Example: {mean} ({sd})</t>
         </r>
       </text>
     </comment>
@@ -502,8 +758,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">With group_page = TRUE: the column whose values each start a page (plan_paginate_group(col = )); blank: the outermost row key.
-Example: PARAM</t>
+          <t xml:space="preserve">Decimals of a token with no format, a comma between tokens; blank: plan_digits().
+Example: 2,3</t>
         </r>
       </text>
     </comment>
@@ -515,255 +771,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">How groups print (plan_row_group(mode = )): value / indent / ...; blank: the default.
-Example: indent</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE, or the columns (names or positions, | between them) whose repeated values print once (plan_row_group(collapse = )); blank: none.
-Example: 1 | 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: one page per value of group_col (plan_paginate_group()); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: with group_page, FALSE leaves the group column unprinted (plan_paginate_group(keep = )); blank: TRUE.
-Example: FALSE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Where blank rows go: a named rule such as between_groups (plan_blanks(where = )); blank: none.
-Example: between_groups</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: a blank row before the first row (plan_blanks(first = )); blank: the default.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: a blank row after the last row (plan_blanks(last = )); blank: the default.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: blank rows count towards pages_max_rows (plan_blanks(counted = )); blank: the default.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The row-key columns folded into one stub column, | between them (plan_stub(vars = )); blank: the row keys.
-Example: group1 | label</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The stub column's name (plan_stub(name = )); blank: the default.
-Example: row_label</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Spaces a level is indented in the stub, a whole number (plan_stub(indent = )); blank: the default.
-Example: 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">How a group's summary row shows in the stub (plan_stub(group_summary = )); blank: the default.
-Example: header</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: fold the stub before cell styles and sorting see the rows (plan_stub(before = )); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Value columns a column page, a whole number (plan_paginate_cols(every = )); blank: no column pages.
+          <t xml:space="preserve">Significant digits (wins over digits); blank: none.
 Example: 4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The columns to cut before (names or positions), | between them (plan_paginate_cols(at = )).
-Example: 16 | 29</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Columns printed on every column page (names or positions), | between them (plan_paginate_cols(keep = )); blank: the stub.
-Example: 1 | 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The order the axes nest in, outermost first: group / rows / cols, or across / down (plan_paginate_cols(order = )); | between them; blank: the default.
-Example: across</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">A separator in the column names: one column page per key before it (plan_paginate_cols(cut_by = )).
-Example: ____</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: TRUE puts every column page on page 1's width scale, FALSE keeps each column's width (plan_paginate_cols(fit = )); blank: TRUE.
-Example: FALSE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: FALSE never cuts inside a spanning header cell (plan_paginate_cols(allow_span_break = )); blank: TRUE.
-Example: FALSE</t>
         </r>
       </text>
     </comment>
@@ -798,8 +807,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">A column name, or .values.
-Example: row_label</t>
+          <t xml:space="preserve">Blank: every analysis variable (the rule); a variable: its exception.
+Example: WEIGHTBL</t>
         </r>
       </text>
     </comment>
@@ -811,8 +820,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Relative width (a number; plan_columns(widths = )). Give one to every printed column (.values covers the value columns); blank: rtfreporter's widths.
-Example: 5</t>
+          <t xml:space="preserve">The statistic, as the ARD names it (mean, sd, median, p ...).
+Example: mean</t>
         </r>
       </text>
     </comment>
@@ -824,34 +833,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE: a row-title column (plan_columns(row_title = )); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: align the decimal points (plan_columns(decimal = )); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: used, not printed (plan_hide()); blank: FALSE.
-Example: TRUE</t>
+          <t xml:space="preserve">Its decimals, a whole number (p, a percent: 1 prints 61.6).
+Example: 1</t>
         </r>
       </text>
     </comment>
@@ -886,8 +869,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The table's rules: tfl (header top and bottom, a bottom rule on the last row) or none; blank: tfl.
-Example: tfl</t>
+          <t xml:space="preserve">Rows a page (plan_paginate_rows(max_rows = )), a whole number; blank: as_rtftables()' default.
+Example: 26</t>
         </r>
       </text>
     </comment>
@@ -899,167 +882,167 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE: realign n (xx.x) count / percent cells to one width; blank: FALSE.
+          <t xml:space="preserve">How a page break may cut: group_safe / group_force / rows / ... (plan_paginate_rows(split = )); blank: as_rtftables()' default.
+Example: group_force</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Row positions to cut before, | between them, with pages_split = rows (plan_paginate_rows(break_before = )); blank: none.
+Example: 20 | 40</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Rows of a group kept together at the foot of a page, a whole number (plan_paginate_rows(min_group_rows = )); blank: the default.
+Example: 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Appended to a group label continued on the next page (plan_paginate_rows(cont_label = )); quote it to keep leading spaces; blank: none.
+Example: " (Cont.)"</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">BY pages: the column(s) whose value partitions the body first, each value a page, the row budget then applying within one (plan_paginate_rows(page_by = )); | between them; print it or hide it (columns$hide); blank: none.
+Example: APERIODC</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">With group_page = TRUE: the column whose values each start a page (plan_paginate_group(col = )); blank: the outermost row key.
+Example: PARAM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">How groups print (plan_row_group(mode = )): value / indent / ...; blank: the default.
+Example: indent</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE, or the columns (names or positions, | between them) whose repeated values print once (plan_row_group(collapse = )); blank: none.
+Example: 1 | 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: one page per value of group_col (plan_paginate_group()); blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: size each column to its widest content (plan_columns(auto_width = )); an explicit rel_width wins; blank: FALSE.
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: with group_page, FALSE leaves the group column unprinted (plan_paginate_group(keep = )); blank: TRUE.
+Example: FALSE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Where blank rows go: a named rule such as between_groups, or row positions -- a blank after each, 0 before the first row, -1 after the last (0 | 5 | -1) (plan_blanks(where = )); blank: none.
+Example: between_groups</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: a blank row before the first row (plan_blanks(first = )); blank: the default.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Data row height in twips (1/1440 inch); blank: from the font size.
-Example: 240</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: TRUE exact (clipped), FALSE at least; blank: FALSE.
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: a blank row after the last row (plan_blanks(last = )); blank: the default.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Column-header row height in twips; blank: row_height_twips.
-Example: 300</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Blank separator row height in twips; blank: row_height_twips.
-Example: 120</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Left cell padding in twips; blank: 0.
-Example: 60</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Right cell padding in twips; blank: 0.
-Example: 60</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Font family of the table; blank: the document's (Courier).
-Example: Arial</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Font size in half-points (18 = 9 pt); blank: the document's.
-Example: 16</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Placement of the table: left / center / right; blank: left.
-Example: center</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Vertical alignment in a cell: bottom / top / center; blank: bottom.
-Example: top</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Cell-text markup, one of script (^{} _{} as super / subscript), relational (&gt;= &lt;= as symbols), all, none; blank: the document's (script).
-Example: all</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
@@ -1068,8 +1051,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">One of detect (an all-empty data row prints as one blank row), collapse (a run of blank rows prints as one), none; blank: both detect and collapse.
-Example: none</t>
+          <t xml:space="preserve">TRUE / FALSE: blank rows count towards pages_max_rows (plan_blanks(counted = )); blank: the default.
+Example: TRUE</t>
         </r>
       </text>
     </comment>
@@ -1081,8 +1064,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The column header's rules: sides from top | bottom | left | right, or none; blank: border's.
-Example: top | bottom</t>
+          <t xml:space="preserve">The row-key columns folded into one stub column, | between them (plan_stub(vars = )); blank: the row keys.
+Example: group1 | label</t>
         </r>
       </text>
     </comment>
@@ -1094,8 +1077,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The spanning header cells' rules: sides, or none; blank: border's.
-Example: bottom</t>
+          <t xml:space="preserve">The stub column's name (plan_stub(name = )); blank: the default.
+Example: row_label</t>
         </r>
       </text>
     </comment>
@@ -1107,8 +1090,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The body rows' rules: sides, or none; blank: border's.
-Example: none</t>
+          <t xml:space="preserve">Spaces a level is indented in the stub, a whole number (plan_stub(indent = )); blank: the default.
+Example: 2</t>
         </r>
       </text>
     </comment>
@@ -1120,8 +1103,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The first body row's rules: sides, or none; blank: border's.
-Example: top</t>
+          <t xml:space="preserve">How a group's summary row shows in the stub (plan_stub(group_summary = )); blank: the default.
+Example: header</t>
         </r>
       </text>
     </comment>
@@ -1133,8 +1116,99 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The last body row's rules: sides, or none; blank: border's.
-Example: bottom</t>
+          <t xml:space="preserve">TRUE / FALSE: fold the stub before cell styles and sorting see the rows (plan_stub(before = )); blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Value columns a column page, a whole number (plan_paginate_cols(every = )); blank: no column pages.
+Example: 4</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The columns to cut before (names or positions), | between them (plan_paginate_cols(at = )).
+Example: 16 | 29</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Columns printed on every column page (names or positions), | between them (plan_paginate_cols(keep = )); blank: the stub.
+Example: 1 | 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The order the axes nest in, outermost first: group / rows / cols, or across / down (plan_paginate_cols(order = )); | between them; blank: the default.
+Example: across</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">A separator in the column names: one column page per key before it (plan_paginate_cols(cut_by = )).
+Example: ____</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: TRUE puts every column page on page 1's width scale, FALSE keeps each column's width (plan_paginate_cols(fit = )); blank: TRUE.
+Example: FALSE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: FALSE never cuts inside a spanning header cell (plan_paginate_cols(allow_span_break = )); blank: TRUE.
+Example: FALSE</t>
         </r>
       </text>
     </comment>
@@ -1169,8 +1243,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The columns styled, | between them (.values = every value column); blank: every column.
-Example: Placebo | .values</t>
+          <t xml:space="preserve">A column name, or .values.
+Example: row_label</t>
         </r>
       </text>
     </comment>
@@ -1182,24 +1256,24 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE: TRUE styles the column header instead of the body; blank: FALSE.
+          <t xml:space="preserve">Relative width (a number; plan_columns(widths = )). Give one to every printed column (.values covers the value columns); blank: rtfreporter's widths.
+Example: 5</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: a row-title column (plan_columns(row_title = )); blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">An R condition over the table's columns choosing the rows; blank: every row. Two rows with a where may not set the same look: join their conditions with |.
-Example: label == "Any TEAE"</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
@@ -1208,7 +1282,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+          <t xml:space="preserve">TRUE / FALSE: align the decimal points (plan_columns(decimal = )); blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
@@ -1221,47 +1295,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+          <t xml:space="preserve">TRUE / FALSE: used, not printed (plan_hide()); blank: FALSE.
 Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">left / center / right; blank: unchanged.
-Example: center</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Text colour, #RRGGBB; blank: unchanged.
-Example: #CC0000</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Cell shading, #RRGGBB; blank: unchanged.
-Example: #EEEEEE</t>
         </r>
       </text>
     </comment>
@@ -1296,8 +1331,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The header row, a whole number (1 = the top).
-Example: 1</t>
+          <t xml:space="preserve">The table's rules: tfl (header top and bottom, a bottom rule on the last row) or none; blank: tfl.
+Example: tfl</t>
         </r>
       </text>
     </comment>
@@ -1309,8 +1344,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The columns the cell sits on: a name, .values (every value column), a position or range (3, 3:31, 3:last), or KEY = value (the columns whose key has that value); | between them.
-Example: .values</t>
+          <t xml:space="preserve">TRUE / FALSE: realign n (xx.x) count / percent cells to one width; blank: FALSE.
+Example: TRUE</t>
         </r>
       </text>
     </comment>
@@ -1322,8 +1357,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Blank: one cell over cols; each: one cell a column; a key's name: one cell per value of that key (a spanner).
-Example: TR01AG1</t>
+          <t xml:space="preserve">TRUE / FALSE: size each column to its widest content (plan_columns(auto_width = )); an explicit rel_width wins; blank: FALSE.
+Example: TRUE</t>
         </r>
       </text>
     </comment>
@@ -1335,8 +1370,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">What prints; a line break is Alt+Enter or \n. Tokens: {col} {col1} {col2} (the column's keys), {n} {n1} {n2} (the population at that depth, read from the ARD), {n:sum} (the total over the cell's columns). Quote it to keep leading spaces.
-Example: {col1}\n(N={n:sum})</t>
+          <t xml:space="preserve">Data row height in twips (1/1440 inch); blank: from the font size.
+Example: 240</t>
         </r>
       </text>
     </comment>
@@ -1348,47 +1383,346 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">left / center / right (col_cell()); blank: the default.
+          <t xml:space="preserve">TRUE / FALSE: TRUE exact (clipped), FALSE at least; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Column-header row height in twips; blank: row_height_twips.
+Example: 300</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Blank separator row height in twips; blank: row_height_twips.
+Example: 120</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Left cell padding in twips; blank: 0.
+Example: 60</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Right cell padding in twips; blank: 0.
+Example: 60</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Font family of the table; blank: the document's (Courier).
+Example: Arial</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Font size in half-points (18 = 9 pt); blank: the document's.
+Example: 16</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Placement of the table: left / center / right; blank: left.
 Example: center</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE; blank: FALSE.
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Vertical alignment in a cell: bottom / top / center; blank: bottom.
+Example: top</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Cell-text markup, one of script (^{} _{} as super / subscript), relational (&gt;= &lt;= as symbols), all, none; blank: the document's (script).
+Example: all</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">One of detect (an all-empty data row prints as one blank row), collapse (a run of blank rows prints as one), none; blank: both detect and collapse.
+Example: none</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The column header's rules: sides from top | bottom | left | right, or none; blank: border's.
+Example: top | bottom</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The spanning header cells' rules: sides, or none; blank: border's.
+Example: bottom</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The body rows' rules: sides, or none; blank: border's.
+Example: none</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The first body row's rules: sides, or none; blank: border's.
+Example: top</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The last body row's rules: sides, or none; blank: border's.
+Example: bottom</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The whole column header's alignment: left / center / right (rtf_table_style()); blank: each column's.
+Example: center</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the whole column header bold; blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The cell's top rule: single / double / none ... (rtf_border()); blank: the header's.
-Example: single</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The cell's bottom rule, as border_top.
-Example: single</t>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the whole column header italic; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The body's default alignment: left / center / right (rtf_table_style()); blank: row-title columns left, the others center.
+Example: left</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the body bold by default; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the body italic by default; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the body underlined by default; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The table's width in twips (1/1440 inch); blank: the page's writable width.
+Example: 12960</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The table's width as a percentage of the page width; blank: the page's writable width.
+Example: 80</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The table's width as a percentage of the writable width (inside the margins); blank: 100.
+Example: 90</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The column header text's alignment, every header row: left / center / right (plan_col_header(col_header_align = )); blank: each column's data alignment.
+Example: center</t>
         </r>
       </text>
     </comment>
@@ -1397,7 +1731,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1447,7 +1781,7 @@
     <t xml:space="preserve">AE</t>
   </si>
   <si>
-    <t xml:space="preserve">TR01AG1 | SEROSTAT</t>
+    <t xml:space="preserve">TRTA | SEX</t>
   </si>
   <si>
     <t xml:space="preserve">group1 = AEBODSYS</t>
@@ -1459,7 +1793,7 @@
     <t xml:space="preserve">.overall | group1 | .depth | -n | label</t>
   </si>
   <si>
-    <t xml:space="preserve">TEAE by SOC / PT, frequency descending</t>
+    <t xml:space="preserve">TEAEs by SOC and PT; the most frequent first within a SOC</t>
   </si>
   <si>
     <t xml:space="preserve">variable</t>
@@ -1471,16 +1805,19 @@
     <t xml:space="preserve">levels</t>
   </si>
   <si>
-    <t xml:space="preserve">TR01AG1</t>
+    <t xml:space="preserve">empty_levels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRTA</t>
   </si>
   <si>
     <t xml:space="preserve">Placebo | Xanomeline Low Dose | Xanomeline High Dose</t>
   </si>
   <si>
-    <t xml:space="preserve">SEROSTAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Positive | Negative</t>
+    <t xml:space="preserve">SEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F | M</t>
   </si>
   <si>
     <t xml:space="preserve">context</t>
@@ -1504,6 +1841,9 @@
     <t xml:space="preserve">{n:.0f} ({p:.1f%})</t>
   </si>
   <si>
+    <t xml:space="preserve">statistic</t>
+  </si>
+  <si>
     <t xml:space="preserve">pages_max_rows</t>
   </si>
   <si>
@@ -1519,6 +1859,9 @@
     <t xml:space="preserve">pages_cont_label</t>
   </si>
   <si>
+    <t xml:space="preserve">pages_page_by</t>
+  </si>
+  <si>
     <t xml:space="preserve">group_col</t>
   </si>
   <si>
@@ -1582,7 +1925,7 @@
     <t xml:space="preserve">colpages_allow_span_break</t>
   </si>
   <si>
-    <t xml:space="preserve">25</t>
+    <t xml:space="preserve">28</t>
   </si>
   <si>
     <t xml:space="preserve">group_force</t>
@@ -1612,13 +1955,13 @@
     <t xml:space="preserve">hide</t>
   </si>
   <si>
-    <t xml:space="preserve">40</t>
+    <t xml:space="preserve">36</t>
   </si>
   <si>
     <t xml:space="preserve">.values</t>
   </si>
   <si>
-    <t xml:space="preserve">10</t>
+    <t xml:space="preserve">8</t>
   </si>
   <si>
     <t xml:space="preserve">border</t>
@@ -1681,7 +2024,40 @@
     <t xml:space="preserve">border_last_row</t>
   </si>
   <si>
-    <t xml:space="preserve">210</t>
+    <t xml:space="preserve">header_align</t>
+  </si>
+  <si>
+    <t xml:space="preserve">header_bold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">header_italic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">align</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">italic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">underline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">table_width_twips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">table_width_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">table_width_pct_of_writable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">col_header_align</t>
+  </si>
+  <si>
+    <t xml:space="preserve">220</t>
   </si>
   <si>
     <t xml:space="preserve">header</t>
@@ -1690,21 +2066,15 @@
     <t xml:space="preserve">where</t>
   </si>
   <si>
-    <t xml:space="preserve">bold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">italic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">align</t>
-  </si>
-  <si>
     <t xml:space="preserve">color</t>
   </si>
   <si>
     <t xml:space="preserve">background</t>
   </si>
   <si>
+    <t xml:space="preserve">indent_twips</t>
+  </si>
+  <si>
     <t xml:space="preserve">line</t>
   </si>
   <si>
@@ -1723,32 +2093,25 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">{col1}
-(N={n:sum})
- n (%)</t>
+    <t xml:space="preserve">{col1} (N={n:sum})</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">single</t>
-  </si>
-  <si>
-    <t xml:space="preserve">none</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System Organ Class
-   Preferred Term</t>
+    <t xml:space="preserve">System organ class
+  Preferred term</t>
   </si>
   <si>
     <t xml:space="preserve">each</t>
   </si>
   <si>
     <t xml:space="preserve">{col2}
-(N={n})</t>
+(N={n})
+n (%)</t>
   </si>
   <si>
     <t xml:space="preserve">spec_version</t>
@@ -2110,18 +2473,186 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G1" t="s">
+        <v>100</v>
+      </c>
+      <c r="H1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I1" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>119</v>
+      </c>
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4"/>
+      <c r="E4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E5" t="s">
+        <v>125</v>
+      </c>
+      <c r="F5"/>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2227,32 +2758,37 @@
       <c r="E1" t="s">
         <v>23</v>
       </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>25</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="F2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="F3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2274,37 +2810,14 @@
         <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G2"/>
-      <c r="H2"/>
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2323,130 +2836,40 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K1" t="s">
-        <v>44</v>
-      </c>
-      <c r="L1" t="s">
-        <v>45</v>
-      </c>
-      <c r="M1" t="s">
-        <v>46</v>
-      </c>
-      <c r="N1" t="s">
-        <v>47</v>
-      </c>
-      <c r="O1" t="s">
-        <v>48</v>
-      </c>
-      <c r="P1" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>50</v>
-      </c>
-      <c r="R1" t="s">
-        <v>51</v>
-      </c>
-      <c r="S1" t="s">
-        <v>52</v>
-      </c>
-      <c r="T1" t="s">
-        <v>53</v>
-      </c>
-      <c r="U1" t="s">
-        <v>54</v>
-      </c>
-      <c r="V1" t="s">
-        <v>55</v>
-      </c>
-      <c r="W1" t="s">
-        <v>56</v>
-      </c>
-      <c r="X1" t="s">
-        <v>57</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" t="s">
-        <v>62</v>
-      </c>
+      <c r="B2"/>
+      <c r="C2"/>
       <c r="D2"/>
       <c r="E2"/>
-      <c r="F2"/>
+      <c r="F2" t="s">
+        <v>35</v>
+      </c>
       <c r="G2"/>
       <c r="H2"/>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2" t="s">
-        <v>63</v>
-      </c>
-      <c r="M2" t="s">
-        <v>64</v>
-      </c>
-      <c r="N2" t="s">
-        <v>64</v>
-      </c>
-      <c r="O2" t="s">
-        <v>64</v>
-      </c>
-      <c r="P2"/>
-      <c r="Q2" t="s">
-        <v>65</v>
-      </c>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2" t="s">
-        <v>64</v>
-      </c>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2465,48 +2888,14 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3"/>
-      <c r="E3"/>
-      <c r="F3"/>
+        <v>33</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2525,77 +2914,316 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="C1" t="s">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="G1" t="s">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="I1" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="J1" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="K1" t="s">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="L1" t="s">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="M1" t="s">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="N1" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="O1" t="s">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="P1" t="s">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="R1" t="s">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="S1" t="s">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="T1" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="U1" t="s">
-        <v>93</v>
+        <v>56</v>
+      </c>
+      <c r="V1" t="s">
+        <v>57</v>
+      </c>
+      <c r="W1" t="s">
+        <v>58</v>
+      </c>
+      <c r="X1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q2"/>
+      <c r="R2" t="s">
+        <v>68</v>
+      </c>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2" t="s">
+        <v>67</v>
+      </c>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L1" t="s">
+        <v>87</v>
+      </c>
+      <c r="M1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N1" t="s">
+        <v>89</v>
+      </c>
+      <c r="O1" t="s">
+        <v>90</v>
+      </c>
+      <c r="P1" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>92</v>
+      </c>
+      <c r="R1" t="s">
+        <v>93</v>
+      </c>
+      <c r="S1" t="s">
+        <v>94</v>
+      </c>
+      <c r="T1" t="s">
+        <v>95</v>
+      </c>
+      <c r="U1" t="s">
+        <v>96</v>
+      </c>
+      <c r="V1" t="s">
+        <v>97</v>
+      </c>
+      <c r="W1" t="s">
+        <v>98</v>
+      </c>
+      <c r="X1" t="s">
+        <v>99</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>101</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>102</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>
@@ -2613,206 +3241,17 @@
       <c r="S2"/>
       <c r="T2"/>
       <c r="U2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-  <legacyDrawing r:id="rIdvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" t="s">
-        <v>99</v>
-      </c>
-      <c r="H1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-  <legacyDrawing r:id="rIdvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H1" t="s">
-        <v>105</v>
-      </c>
-      <c r="I1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5" t="s">
-        <v>110</v>
-      </c>
-      <c r="I5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C6" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6"/>
-      <c r="E6" t="s">
-        <v>113</v>
-      </c>
-      <c r="F6"/>
-      <c r="G6"/>
-      <c r="H6"/>
-      <c r="I6"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D7" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" t="s">
-        <v>115</v>
-      </c>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Samples on the onco data: ard-spec workbooks, spec-yaml fixture, the onco example study
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01218WKStb6ChPBdfjbCjefs
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -265,7 +265,7 @@
             <name val="Tahoma"/>
           </rPr>
           <t xml:space="preserve">Blank: one cell over cols; each: one cell a column; a key's name: one cell per value of that key (a spanner).
-Example: TR01AG1</t>
+Example: TRTA</t>
         </r>
       </text>
     </comment>
@@ -366,7 +366,7 @@
             <name val="Tahoma"/>
           </rPr>
           <t xml:space="preserve">The key spread across the columns, outermost first, | between them (table_plan(cols = )).
-Example: TRT01A | SEROSTAT</t>
+Example: TRTA | SEX</t>
         </r>
       </text>
     </comment>
@@ -443,8 +443,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE, FALSE, or the sort keys in order, - in front for descending (plan_sort()); blank: the data's order.
-Example: .overall | group1 | -n | label</t>
+          <t xml:space="preserve">TRUE, FALSE, or the sort keys in order, - in front for descending (plan_sort()): a column, .overall, .depth, a statistic (summed over the columns), stat[col] for one column (-n[Total]), stat@key for a group's own count carried to its rows (-n@group1: SOCs by their own count); blank: the data's order.
+Example: .overall | -n@group1 | group1 | -n | label</t>
         </r>
       </text>
     </comment>
@@ -482,12 +482,194 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Which population {n} in the column header is, for a table split by page (a lab parameter): page (those with that page's data), table (the analysis set), or both as n = page | N = table for {n} and {N}; blank: page (warns when both exist and differ). Both must be in the ARD.
+          <t xml:space="preserve">Which population {n} in the column header is, for a table split by page (a lab parameter): page (those with that page's data), table (the population), or both as n = page | N = table for {n} and {N}; blank: page (warns when both exist and differ). Both must be in the ARD.
 Example: n = page | N = table</t>
         </r>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The heading of a Total column (plan_total()): the ARD's overall rows, its analyses run again without their by (analyses$overall), as one more column; its {n} is the study total. Blank: none.
+Example: Total</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Where the Total column goes among the column key's values: last or first; blank: last.
+Example: first</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The row of a hierarchy's overall counts (a hierarchical analysis with args over_variables = TRUE) and what it prints: normalize_ard(overall = ), written by tfl_normalize_code(). Blank: no such row.
+Example: Subjects with at least one TEAE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">One record's statistics (the same analysis and keys) in named groups (plan_stat_groups()): | between groups, a comma between a group's statistics. The key .stat_group then names them in cols (TRT01A | .stat_group: N in one column, the rate and CI in the next) or in rows (one group under another, in the order said); a cells row's variable may be a group's name, its template one row or several. The ARD stays as it is: no relabelled variable. .variables = RESP limits the groups to those variables, and .others = n puts the other variables' records whole in that group (a subgroup's own n (%) beside its ORR). Blank: none.
+Example: n = N | orr_ci = n, estimate, conf.low, conf.high</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Subgroups as one pair of keys: name = its layers, a comma between them, * crossing variables (AGEGR1 * SEX), | between several keys; or the strata slots (subgroup = group2, group3) (normalize_ard(stack = ), written by tfl_normalize_code()). rows then names subgroup and subgroup_level, whatever group slot each variable came in. Blank: none.
+Example: subgroup = ALL, SEX, AGEGR1, AGEGR1 * SEX</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">What joins a crossed layer's names and levels (AGEGR1 / SEX, 65-80 / F) (normalize_ard(stack_sep = )). Blank: ' / '.
+Example:  x </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE: a crossed layer's outer levels in a key of their own, subgroup_outer, its innermost in subgroup_level, so rows grp = subgroup | outer = subgroup_outer | lvl = subgroup_level with a stub prints the outer level as a heading (normalize_ard(stack_nest = )). Blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Comparison columns: their names, | between them (plan_compare()). Each reads the ARD's comparison records (a test's p-value, a difference and its CI: the column key with no value) and puts them on the row of their variable; its templates are the cells rows whose variable is the column's name. Blank: none.
+Example: p | diff</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The column that splits the comparisons into columns, one a level (plan_compare(by = )): each active arm against placebo. Blank: one comparison a variable.
+Example: COMPARISON</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Where the comparison columns go: last (blank) or first (plan_compare(position = )).
+Example: first</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Row keys the table also shows as variables, | between them: their own counts (the subgroup variable tabulated by arm) stay in the body, a block of their own beside the subgroup layer of another analysis (table_plan(show_keys = )). Blank: none.
+Example: SEX | AGEGR1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Rows kept by a condition over the record (plan_filter()): one R condition over its statistics and keys, as a cells row's when (p &gt;= 0.05); several joined by &amp;. A SOC stays when one of its PTs does; the overall row always stays. Blank: every row.
+Example: p &gt;= 0.05</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the condition in any column (TRUE, blank) or every column (FALSE) (plan_filter(any = )).
+Example: FALSE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">keep (blank): a parent row (a SOC) stays exactly when one of its children does; drop: judged by its own counts (plan_filter(parents = )).
+Example: drop</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -587,6 +769,19 @@
         </r>
       </text>
     </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Its rows under one level of another variable: that variable, a colon, the level as the table shows it (plan_nest()); after that row, one indent deeper, its own heading dropped; blank: its own block.
+Example: RACE: Asian</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -947,12 +1142,25 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">With pages_page_by (one column): each BY page's name from a template, as group_heading: {value} the page's value, {n} its N as the ARD states it (plan_paginate_rows(heading = )); blank: the value.
+Example: Treatment: {value} (N={n})</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">With group_page = TRUE: the column whose values each start a page (plan_paginate_group(col = )); blank: the outermost row key.
 Example: PARAM</t>
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -965,7 +1173,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -978,7 +1186,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -991,7 +1199,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1004,7 +1212,20 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">With group_page = TRUE: each page's name, the heading rtf_tables(auto_section = TRUE) prints, from a template: {value} the page's value, {n} its N as the ARD states it (the page variable's own tabulation, cards::ard_tabulate(adsl, variables = TRT01A)) (plan_paginate_group(heading = )); blank: the value.
+Example: Treatment: {value} (N={n})</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1017,7 +1238,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1030,7 +1251,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1043,7 +1264,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1056,7 +1277,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1069,7 +1290,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1082,7 +1303,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1095,7 +1316,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1108,7 +1329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1121,7 +1342,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1134,7 +1355,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1147,7 +1368,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1160,7 +1381,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1173,7 +1394,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1186,7 +1407,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1199,7 +1420,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AD1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1731,7 +1952,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1775,13 +1996,55 @@
     <t xml:space="preserve">header_n</t>
   </si>
   <si>
+    <t xml:space="preserve">total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total_position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">overall_label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stat_groups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stack_sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stack_nest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compare_by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compare_position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">show_keys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep_where</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep_any</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep_parents</t>
+  </si>
+  <si>
     <t xml:space="preserve">note</t>
   </si>
   <si>
     <t xml:space="preserve">AE</t>
   </si>
   <si>
-    <t xml:space="preserve">TRTA | SEX</t>
+    <t xml:space="preserve">TRT01A | SEX</t>
   </si>
   <si>
     <t xml:space="preserve">group1 = AEBODSYS</t>
@@ -1808,10 +2071,13 @@
     <t xml:space="preserve">empty_levels</t>
   </si>
   <si>
-    <t xml:space="preserve">TRTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placebo | Xanomeline Low Dose | Xanomeline High Dose</t>
+    <t xml:space="preserve">under</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRT01A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drug X | Control</t>
   </si>
   <si>
     <t xml:space="preserve">SEX</t>
@@ -1862,6 +2128,9 @@
     <t xml:space="preserve">pages_page_by</t>
   </si>
   <si>
+    <t xml:space="preserve">pages_heading</t>
+  </si>
+  <si>
     <t xml:space="preserve">group_col</t>
   </si>
   <si>
@@ -1875,6 +2144,9 @@
   </si>
   <si>
     <t xml:space="preserve">group_keep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">group_heading</t>
   </si>
   <si>
     <t xml:space="preserve">blank_where</t>
@@ -2479,31 +2751,31 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="D1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="E1" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="F1" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="G1" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="H1" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="I1" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J1" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="K1" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2523,39 +2795,39 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="E1" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="F1" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="G1" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="H1" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="I1" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2566,40 +2838,40 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
       <c r="H3"/>
       <c r="I3" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
@@ -2608,19 +2880,19 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="E5" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="F5"/>
       <c r="G5"/>
@@ -2649,10 +2921,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2703,31 +2975,87 @@
       <c r="L1" t="s">
         <v>14</v>
       </c>
+      <c r="M1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+      <c r="R1" t="s">
+        <v>20</v>
+      </c>
+      <c r="S1" t="s">
+        <v>21</v>
+      </c>
+      <c r="T1" t="s">
+        <v>22</v>
+      </c>
+      <c r="U1" t="s">
+        <v>23</v>
+      </c>
+      <c r="V1" t="s">
+        <v>24</v>
+      </c>
+      <c r="W1" t="s">
+        <v>25</v>
+      </c>
+      <c r="X1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
       <c r="K2"/>
-      <c r="L2" t="s">
-        <v>20</v>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2747,48 +3075,53 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>38</v>
+      </c>
+      <c r="G1" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="F2"/>
+      <c r="G2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="F3"/>
+      <c r="G3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2807,7 +3140,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2816,7 +3149,7 @@
         <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2836,37 +3169,37 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="H1" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2"/>
       <c r="F2" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="G2"/>
       <c r="H2"/>
@@ -2888,13 +3221,13 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2914,96 +3247,102 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="F1" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G1" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="H1" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="I1" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="J1" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K1" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="L1" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="M1" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="N1" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="O1" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="P1" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="Q1" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="R1" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="S1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="T1" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="U1" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="V1" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="W1" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="X1" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="Y1" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="Z1" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="AA1" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AB1" t="s">
-        <v>63</v>
+        <v>78</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -3014,34 +3353,36 @@
       <c r="J2"/>
       <c r="K2"/>
       <c r="L2"/>
-      <c r="M2" t="s">
-        <v>66</v>
-      </c>
-      <c r="N2" t="s">
-        <v>67</v>
-      </c>
+      <c r="M2"/>
+      <c r="N2"/>
       <c r="O2" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="P2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q2"/>
+        <v>84</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>84</v>
+      </c>
       <c r="R2" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="S2"/>
-      <c r="T2"/>
-      <c r="U2" t="s">
-        <v>67</v>
-      </c>
+      <c r="T2" t="s">
+        <v>85</v>
+      </c>
+      <c r="U2"/>
       <c r="V2"/>
-      <c r="W2"/>
+      <c r="W2" t="s">
+        <v>84</v>
+      </c>
       <c r="X2"/>
       <c r="Y2"/>
       <c r="Z2"/>
       <c r="AA2"/>
       <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3060,30 +3401,30 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="D1" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="E1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="F1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -3091,13 +3432,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -3120,110 +3461,110 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="F1" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="G1" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="H1" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="I1" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="J1" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="K1" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="L1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="M1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="N1" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="O1" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="P1" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="Q1" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="R1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="S1" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="T1" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="U1" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="V1" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="W1" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="X1" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="Y1" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="Z1" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="AA1" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AB1" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AC1" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="AD1" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="AE1" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="AF1" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>

</xml_diff>